<commit_message>
V5  VSL Solver (Fall Analysis)
V5 has energy absorption from falling and better spring outputs
</commit_message>
<xml_diff>
--- a/users/jonathan-xie/experimental-apps/vsl-solver/v4/v4-configs.xlsx
+++ b/users/jonathan-xie/experimental-apps/vsl-solver/v4/v4-configs.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:BW4"/>
+  <dimension ref="A1:BW5"/>
   <sheetFormatPr defaultRowHeight="22"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1573,14 +1573,253 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mason CAD (205.3mm Legs) </t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Use VSL</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Use VSL</t>
+        </is>
+      </c>
+      <c r="E5" s="4">
+        <v>46318.060309837965</v>
+      </c>
+      <c r="F5" s="3">
+        <v>8.75</v>
+      </c>
+      <c r="G5" s="3">
+        <v>200</v>
+      </c>
+      <c r="H5" s="3">
+        <v>200</v>
+      </c>
+      <c r="I5" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="J5" s="3">
+        <v>20</v>
+      </c>
+      <c r="K5" s="3">
+        <v>272.88249263865174</v>
+      </c>
+      <c r="L5" s="3">
+        <v>6</v>
+      </c>
+      <c r="M5" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="N5" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="O5" s="3">
+        <v>8.75</v>
+      </c>
+      <c r="P5" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="3">
+        <v>0</v>
+      </c>
+      <c r="R5" s="3">
+        <v>0</v>
+      </c>
+      <c r="S5" s="3">
+        <v>0</v>
+      </c>
+      <c r="T5" s="3">
+        <v>9.81</v>
+      </c>
+      <c r="U5" s="3">
+        <v>50</v>
+      </c>
+      <c r="V5" s="3">
+        <v>25</v>
+      </c>
+      <c r="W5" s="3">
+        <v>35</v>
+      </c>
+      <c r="X5" s="3">
+        <v>35</v>
+      </c>
+      <c r="Y5" s="3">
+        <v>25</v>
+      </c>
+      <c r="Z5" s="3">
+        <v>25</v>
+      </c>
+      <c r="AA5" s="3">
+        <v>200</v>
+      </c>
+      <c r="AB5" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="3">
+        <v>100</v>
+      </c>
+      <c r="AD5" s="3">
+        <v>165</v>
+      </c>
+      <c r="AE5" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF5" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG5" s="3">
+        <v>85.8375</v>
+      </c>
+      <c r="AH5" s="3">
+        <v>85.8375</v>
+      </c>
+      <c r="AI5" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yz</t>
+        </is>
+      </c>
+      <c r="AK5" s="3">
+        <v>62.88850811914982</v>
+      </c>
+      <c r="AL5" s="3">
+        <v>80</v>
+      </c>
+      <c r="AM5" s="3">
+        <v>10</v>
+      </c>
+      <c r="AN5" s="3">
+        <v>137.88681177871507</v>
+      </c>
+      <c r="AO5" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP5" s="3">
+        <v>8.418095061266762</v>
+      </c>
+      <c r="AQ5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AR5" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS5" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT5" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU5" s="3">
+        <v>149.27616068766133</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">r_h, p0, S_u</t>
+        </is>
+      </c>
+      <c r="AW5" s="3">
+        <v>8</v>
+      </c>
+      <c r="AX5" s="3">
+        <v>0.015115453537447365</v>
+      </c>
+      <c r="AY5" s="3">
+        <v>27.735715196569537</v>
+      </c>
+      <c r="AZ5" s="3">
+        <v>-27.750830650106984</v>
+      </c>
+      <c r="BA5" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB5" s="3">
+        <v>455.8266719381592</v>
+      </c>
+      <c r="BC5" s="3">
+        <v>155.87549223213014</v>
+      </c>
+      <c r="BD5" s="3">
+        <v>-0.01565360153959716</v>
+      </c>
+      <c r="BE5" s="3">
+        <v>17.1675</v>
+      </c>
+      <c r="BF5" s="3">
+        <v>552.6499900306806</v>
+      </c>
+      <c r="BG5" s="3">
+        <v>686.6997506370908</v>
+      </c>
+      <c r="BH5" s="3">
+        <v>0.054498156727933456</v>
+      </c>
+      <c r="BI5" s="3">
+        <v>-42.885397396080656</v>
+      </c>
+      <c r="BJ5" s="3">
+        <v>0</v>
+      </c>
+      <c r="BK5" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL5" s="3">
+        <v>30</v>
+      </c>
+      <c r="BM5" s="3">
+        <v>0</v>
+      </c>
+      <c r="BN5" s="3">
+        <v>90</v>
+      </c>
+      <c r="BO5" s="3">
+        <v>-100</v>
+      </c>
+      <c r="BP5" s="3">
+        <v>100</v>
+      </c>
+      <c r="BQ5" s="3">
+        <v>0</v>
+      </c>
+      <c r="BR5" s="3">
+        <v>200</v>
+      </c>
+      <c r="BS5" s="3">
+        <v>0</v>
+      </c>
+      <c r="BT5" s="3">
+        <v>200</v>
+      </c>
+      <c r="BU5" s="3">
+        <v>-100</v>
+      </c>
+      <c r="BV5" s="3">
+        <v>100</v>
+      </c>
+      <c r="BW5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">none</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:BW4"/>
+  <autoFilter ref="A1:BW5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="22"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1626,7 +1865,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"dp":1,"name":"8.75 kg baseline","color":"mint","savedAt":"2026-10-22T02:37:20.651Z","snapshot":{"schema":"general-vsl/v4-pulley","torqueConvention":"physical-link2-ccw/v2","ratioConvention":"output-over-input","parameters":{"L2":300,"L3":300,"ra":50,"rb":25,"rc":35,"rd":35,"re":25,"rf":25,"rw":200,"alpha":0,"phi0":0,"te":100,"tc":165,"m1":8.75,"m2":0,"m3":0,"m5":0,"m6":0,"g":9.81,"beta":0,"Fn":85.8375,"Ft":0,"Fy":0,"Fz":85.8375,"loadMode":"yz","Tab0":0,"Tcd0":0,"Tef0":0,"springEnabled":true,"springK":8,"hornR":62.22694951186731,"Sv":100,"rs":10,"p0":330.8692828089511,"nu":0,"Su":9.387776728149294},"driven":{"q23":"q23","qab":"qab","qdc":"qdc","qfe":"qfe"},"springDriven":null,"ranges":{"alpha":{"min":0,"max":30},"beta":{"min":0,"max":90},"Fn":{"min":0,"max":200},"Ft":{"min":-100,"max":100},"Fy":{"min":-100,"max":100},"Fz":{"min":0,"max":200}},"theta2":135,"period":8,"absoluteTorques":false,"fullTravel":false,"clampRanges":true,"view":{"showTau2":true,"showTau4":true,"showWheelForces":true,"showWheel":true,"showAB":true,"showDrive":true},"outputs":{"tau2":-0.020625449196600698,"tauG":36.417766998060166,"tauS":-36.397141548863566,"tau4":0,"Fs":591.8657101337469,"pe":348.73056050174307,"globalMaxTau2":0.06274113617364208,"globalMaxTau4":17.1675,"globalMaxFs":848.4898544049762,"globalMaxTab":994.9518973690548,"globalMaxDz":435.5932247458122,"compensationError":-0.056635677848393406,"zeta":-53.305793287305484,"zetaApplied":0},"springDriving":{"springK":true,"hornR":false,"Sv":true,"rs":true,"p0":false,"nu":true,"Su":false}}}</t>
+          <t xml:space="preserve">{"dp":1,"name":"8.75 kg baseline","color":"mint","savedAt":"2026-10-22T02:37:20.651000Z","snapshot":{"schema":"general-vsl/v4-pulley","torqueConvention":"physical-link2-ccw/v2","ratioConvention":"output-over-input","parameters":{"L2":300,"L3":300,"ra":50,"rb":25,"rc":35,"rd":35,"re":25,"rf":25,"rw":200,"alpha":0,"phi0":0,"te":100,"tc":165,"m1":8.75,"m2":0,"m3":0,"m5":0,"m6":0,"g":9.81,"beta":0,"Fn":85.8375,"Ft":0,"Fy":0,"Fz":85.8375,"loadMode":"yz","Tab0":0,"Tcd0":0,"Tef0":0,"springEnabled":true,"springK":8,"hornR":62.22694951186731,"Sv":100,"rs":10,"p0":330.8692828089511,"nu":0,"Su":9.387776728149294},"driven":{"q23":"q23","qab":"qab","qdc":"qdc","qfe":"qfe"},"springDriven":null,"ranges":{"alpha":{"min":0,"max":30},"beta":{"min":0,"max":90},"Fn":{"min":0,"max":200},"Ft":{"min":-100,"max":100},"Fy":{"min":-100,"max":100},"Fz":{"min":0,"max":200}},"theta2":135,"period":8,"absoluteTorques":false,"fullTravel":false,"clampRanges":true,"view":{"showTau2":true,"showTau4":true,"showWheelForces":true,"showWheel":true,"showAB":true,"showDrive":true},"outputs":{"tau2":-0.020625449196600698,"tauG":36.417766998060166,"tauS":-36.397141548863566,"tau4":0,"Fs":591.8657101337469,"pe":348.73056050174307,"globalMaxTau2":0.06274113617364208,"globalMaxTau4":17.1675,"globalMaxFs":848.4898544049762,"globalMaxTab":994.9518973690548,"globalMaxDz":435.5932247458122,"compensationError":-0.056635677848393406,"zeta":-53.305793287305484,"zetaApplied":0},"springDriving":{"springK":true,"hornR":false,"Sv":true,"rs":true,"p0":false,"nu":true,"Su":false}}}</t>
         </is>
       </c>
     </row>
@@ -1638,7 +1877,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"dp":2,"name":"10/22 POR, Alpha = 0","color":"none","savedAt":"2026-10-22T05:11:22.003Z","snapshot":{"schema":"general-vsl/v4-pulley","torqueConvention":"physical-link2-ccw/v2","ratioConvention":"output-over-input","parameters":{"L2":300,"L3":300,"ra":50,"rb":25,"rc":25,"rd":50,"re":35,"rf":70,"rw":200,"alpha":0,"phi0":0,"te":100,"tc":165,"m1":8.75,"m2":0,"m3":0,"m5":0,"m6":0,"g":9.81,"beta":0,"Fn":85.8375,"Ft":0,"Fy":0,"Fz":85.8375,"loadMode":"yz","Tab0":0,"Tcd0":0,"Tef0":0,"springEnabled":true,"springK":6,"hornR":81.0181311351,"Sv":100,"rs":10,"p0":152.46505385868363,"nu":0,"Su":8.106024183399995},"driven":{"q23":"q23","qab":"qab","qdc":"rd","qfe":"rf"},"springDriven":null,"springDriving":{"springK":true,"hornR":false,"Sv":true,"rs":true,"p0":false,"nu":true,"Su":false},"ranges":{"alpha":{"min":0,"max":30},"beta":{"min":0,"max":0},"Fn":{"min":0,"max":200},"Ft":{"min":-100,"max":100},"Fy":{"min":-100,"max":100},"Fz":{"min":0,"max":200}},"theta2":103.55504590729112,"period":8,"absoluteTorques":false,"fullTravel":false,"clampRanges":true,"view":{"showTau2":true,"showTau4":true,"showWheelForces":true,"showWheel":true,"showAB":true,"showDrive":true},"visible":{"t3":true,"t5":true,"t6":true,"du":true,"dv":true,"dy":true,"dz":true,"gammaUV":true,"gammaYZ":true},"series":{"t2-torque-tauG":true,"t2-torque-tauS":true,"t2-torque-tau2":true,"t2-torque-tau4":true,"t2-tension-ab":true,"t2-tension-cd":true,"t2-tension-ef":true,"t2-force-F12":true,"t2-force-F14":true,"t2-force-F25":true,"t2-force-F32":true,"t2-force-Fw":true,"dz-torque-tauG":true,"dz-torque-tauS":true,"dz-torque-tau2":true,"dz-torque-tau4":true,"dz-tension-ab":true,"dz-tension-cd":true,"dz-tension-ef":true,"dz-force-F12":true,"dz-force-F14":true,"dz-force-F25":true,"dz-force-F32":true,"dz-force-Fw":true,"beta-torque-tauG":true,"beta-torque-tauS":true,"beta-torque-tau2":true,"beta-torque-tau4":true,"beta-tension-ab":true,"beta-tension-cd":true,"beta-tension-ef":true,"beta-force-F12":true,"beta-force-F14":true,"beta-force-F25":true,"beta-force-F32":true,"beta-force-Fw":true,"alpha-torque-tauG":true,"alpha-torque-tauS":true,"alpha-torque-tau2":true,"alpha-torque-tau4":true,"alpha-tension-ab":true,"alpha-tension-cd":true,"alpha-tension-ef":true,"alpha-force-F12":true,"alpha-force-F14":true,"alpha-force-F25":true,"alpha-force-F32":true,"alpha-force-Fw":true},"outputs":{"tau2":0.017139940185623814,"tauG":12.071127272781894,"tauS":-12.088267212967517,"tau4":0,"Fs":198.97844938180913,"pe":178.22029189381868,"globalMaxTau2":0.017665297379156897,"globalMaxTau4":0,"globalMaxFs":693.1787801958694,"globalMaxTab":994.9518973690548,"globalMaxDz":435.5932247458122,"compensationError":0.14199121422793226,"zeta":-40.3046961390234,"zetaApplied":0}},"outputsStale":false}</t>
+          <t xml:space="preserve">{"dp":2,"name":"10/22 POR, Alpha = 0","color":"none","savedAt":"2026-10-22T05:11:22.003000Z","snapshot":{"schema":"general-vsl/v4-pulley","torqueConvention":"physical-link2-ccw/v2","ratioConvention":"output-over-input","parameters":{"L2":300,"L3":300,"ra":50,"rb":25,"rc":25,"rd":50,"re":35,"rf":70,"rw":200,"alpha":0,"phi0":0,"te":100,"tc":165,"m1":8.75,"m2":0,"m3":0,"m5":0,"m6":0,"g":9.81,"beta":0,"Fn":85.8375,"Ft":0,"Fy":0,"Fz":85.8375,"loadMode":"yz","Tab0":0,"Tcd0":0,"Tef0":0,"springEnabled":true,"springK":6,"hornR":81.0181311351,"Sv":100,"rs":10,"p0":152.46505385868363,"nu":0,"Su":8.106024183399995},"driven":{"q23":"q23","qab":"qab","qdc":"rd","qfe":"rf"},"springDriven":null,"springDriving":{"springK":true,"hornR":false,"Sv":true,"rs":true,"p0":false,"nu":true,"Su":false},"ranges":{"alpha":{"min":0,"max":30},"beta":{"min":0,"max":0},"Fn":{"min":0,"max":200},"Ft":{"min":-100,"max":100},"Fy":{"min":-100,"max":100},"Fz":{"min":0,"max":200}},"theta2":103.55504590729112,"period":8,"absoluteTorques":false,"fullTravel":false,"clampRanges":true,"view":{"showTau2":true,"showTau4":true,"showWheelForces":true,"showWheel":true,"showAB":true,"showDrive":true},"visible":{"t3":true,"t5":true,"t6":true,"du":true,"dv":true,"dy":true,"dz":true,"gammaUV":true,"gammaYZ":true},"series":{"t2-torque-tauG":true,"t2-torque-tauS":true,"t2-torque-tau2":true,"t2-torque-tau4":true,"t2-tension-ab":true,"t2-tension-cd":true,"t2-tension-ef":true,"t2-force-F12":true,"t2-force-F14":true,"t2-force-F25":true,"t2-force-F32":true,"t2-force-Fw":true,"dz-torque-tauG":true,"dz-torque-tauS":true,"dz-torque-tau2":true,"dz-torque-tau4":true,"dz-tension-ab":true,"dz-tension-cd":true,"dz-tension-ef":true,"dz-force-F12":true,"dz-force-F14":true,"dz-force-F25":true,"dz-force-F32":true,"dz-force-Fw":true,"beta-torque-tauG":true,"beta-torque-tauS":true,"beta-torque-tau2":true,"beta-torque-tau4":true,"beta-tension-ab":true,"beta-tension-cd":true,"beta-tension-ef":true,"beta-force-F12":true,"beta-force-F14":true,"beta-force-F25":true,"beta-force-F32":true,"beta-force-Fw":true,"alpha-torque-tauG":true,"alpha-torque-tauS":true,"alpha-torque-tau2":true,"alpha-torque-tau4":true,"alpha-tension-ab":true,"alpha-tension-cd":true,"alpha-tension-ef":true,"alpha-force-F12":true,"alpha-force-F14":true,"alpha-force-F25":true,"alpha-force-F32":true,"alpha-force-Fw":true},"outputs":{"tau2":0.017139940185623814,"tauG":12.071127272781894,"tauS":-12.088267212967517,"tau4":0,"Fs":198.97844938180913,"pe":178.22029189381868,"globalMaxTau2":0.017665297379156897,"globalMaxTau4":0,"globalMaxFs":693.1787801958694,"globalMaxTab":994.9518973690548,"globalMaxDz":435.5932247458122,"compensationError":0.14199121422793226,"zeta":-40.3046961390234,"zetaApplied":0}},"outputsStale":false}</t>
         </is>
       </c>
     </row>
@@ -1650,7 +1889,19 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"dp":3,"name":"10/22 POR, Alpha = 20","color":"none","savedAt":"2026-10-22T05:11:43.602Z","snapshot":{"schema":"general-vsl/v4-pulley","torqueConvention":"physical-link2-ccw/v2","ratioConvention":"output-over-input","parameters":{"L2":300,"L3":300,"ra":50,"rb":25,"rc":25,"rd":50,"re":35,"rf":70,"rw":200,"alpha":20,"phi0":0,"te":100,"tc":165,"m1":8.75,"m2":0,"m3":0,"m5":0,"m6":0,"g":9.81,"beta":0,"Fn":85.8375,"Ft":0,"Fy":0,"Fz":85.8375,"loadMode":"yz","Tab0":0,"Tcd0":0,"Tef0":0,"springEnabled":true,"springK":6,"hornR":76.54191184861334,"Sv":100,"rs":10,"p0":174.9162355946656,"nu":0,"Su":8.500309950238233},"driven":{"q23":"q23","qab":"qab","qdc":"rd","qfe":"rf"},"springDriven":null,"springDriving":{"springK":true,"hornR":false,"Sv":true,"rs":true,"p0":false,"nu":true,"Su":false},"ranges":{"alpha":{"min":0,"max":30},"beta":{"min":0,"max":0},"Fn":{"min":0,"max":200},"Ft":{"min":-100,"max":100},"Fy":{"min":-100,"max":100},"Fz":{"min":0,"max":200}},"theta2":103.55504590729112,"period":8,"absoluteTorques":false,"fullTravel":false,"clampRanges":true,"view":{"showTau2":true,"showTau4":true,"showWheelForces":true,"showWheel":true,"showAB":true,"showDrive":true},"visible":{"t3":true,"t5":true,"t6":true,"du":true,"dv":true,"dy":true,"dz":true,"gammaUV":true,"gammaYZ":true},"series":{"t2-torque-tauG":true,"t2-torque-tauS":true,"t2-torque-tau2":true,"t2-torque-tau4":true,"t2-tension-ab":true,"t2-tension-cd":true,"t2-tension-ef":true,"t2-force-F12":true,"t2-force-F14":true,"t2-force-F25":true,"t2-force-F32":true,"t2-force-Fw":true,"dz-torque-tauG":true,"dz-torque-tauS":true,"dz-torque-tau2":true,"dz-torque-tau4":true,"dz-tension-ab":true,"dz-tension-cd":true,"dz-tension-ef":true,"dz-force-F12":true,"dz-force-F14":true,"dz-force-F25":true,"dz-force-F32":true,"dz-force-Fw":true,"beta-torque-tauG":true,"beta-torque-tauS":true,"beta-torque-tau2":true,"beta-torque-tau4":true,"beta-tension-ab":true,"beta-tension-cd":true,"beta-tension-ef":true,"beta-force-F12":true,"beta-force-F14":true,"beta-force-F25":true,"beta-force-F32":true,"beta-force-Fw":true,"alpha-torque-tauG":true,"alpha-torque-tauS":true,"alpha-torque-tau2":true,"alpha-torque-tau4":true,"alpha-tension-ab":true,"alpha-tension-cd":true,"alpha-tension-ef":true,"alpha-force-F12":true,"alpha-force-F14":true,"alpha-force-F25":true,"alpha-force-F32":true,"alpha-force-Fw":true},"outputs":{"tau2":0.017768093441409505,"tauG":11.343149222800683,"tauS":-11.360917316242093,"tau4":0,"Fs":214.75347736688684,"pe":196.8809358202675,"globalMaxTau2":0.019679624716665955,"globalMaxTau4":0,"globalMaxFs":678.5552779524771,"globalMaxTab":1030.0496259556362,"globalMaxDz":409.3237389579775,"compensationError":0.15664162652204716,"zeta":-43.61013949287524,"zetaApplied":0}},"outputsStale":false}</t>
+          <t xml:space="preserve">{"dp":3,"name":"10/22 POR, Alpha = 20","color":"none","savedAt":"2026-10-22T05:11:43.602000Z","snapshot":{"schema":"general-vsl/v4-pulley","torqueConvention":"physical-link2-ccw/v2","ratioConvention":"output-over-input","parameters":{"L2":300,"L3":300,"ra":50,"rb":25,"rc":25,"rd":50,"re":35,"rf":70,"rw":200,"alpha":20,"phi0":0,"te":100,"tc":165,"m1":8.75,"m2":0,"m3":0,"m5":0,"m6":0,"g":9.81,"beta":0,"Fn":85.8375,"Ft":0,"Fy":0,"Fz":85.8375,"loadMode":"yz","Tab0":0,"Tcd0":0,"Tef0":0,"springEnabled":true,"springK":6,"hornR":76.54191184861334,"Sv":100,"rs":10,"p0":174.9162355946656,"nu":0,"Su":8.500309950238233},"driven":{"q23":"q23","qab":"qab","qdc":"rd","qfe":"rf"},"springDriven":null,"springDriving":{"springK":true,"hornR":false,"Sv":true,"rs":true,"p0":false,"nu":true,"Su":false},"ranges":{"alpha":{"min":0,"max":30},"beta":{"min":0,"max":0},"Fn":{"min":0,"max":200},"Ft":{"min":-100,"max":100},"Fy":{"min":-100,"max":100},"Fz":{"min":0,"max":200}},"theta2":103.55504590729112,"period":8,"absoluteTorques":false,"fullTravel":false,"clampRanges":true,"view":{"showTau2":true,"showTau4":true,"showWheelForces":true,"showWheel":true,"showAB":true,"showDrive":true},"visible":{"t3":true,"t5":true,"t6":true,"du":true,"dv":true,"dy":true,"dz":true,"gammaUV":true,"gammaYZ":true},"series":{"t2-torque-tauG":true,"t2-torque-tauS":true,"t2-torque-tau2":true,"t2-torque-tau4":true,"t2-tension-ab":true,"t2-tension-cd":true,"t2-tension-ef":true,"t2-force-F12":true,"t2-force-F14":true,"t2-force-F25":true,"t2-force-F32":true,"t2-force-Fw":true,"dz-torque-tauG":true,"dz-torque-tauS":true,"dz-torque-tau2":true,"dz-torque-tau4":true,"dz-tension-ab":true,"dz-tension-cd":true,"dz-tension-ef":true,"dz-force-F12":true,"dz-force-F14":true,"dz-force-F25":true,"dz-force-F32":true,"dz-force-Fw":true,"beta-torque-tauG":true,"beta-torque-tauS":true,"beta-torque-tau2":true,"beta-torque-tau4":true,"beta-tension-ab":true,"beta-tension-cd":true,"beta-tension-ef":true,"beta-force-F12":true,"beta-force-F14":true,"beta-force-F25":true,"beta-force-F32":true,"beta-force-Fw":true,"alpha-torque-tauG":true,"alpha-torque-tauS":true,"alpha-torque-tau2":true,"alpha-torque-tau4":true,"alpha-tension-ab":true,"alpha-tension-cd":true,"alpha-tension-ef":true,"alpha-force-F12":true,"alpha-force-F14":true,"alpha-force-F25":true,"alpha-force-F32":true,"alpha-force-Fw":true},"outputs":{"tau2":0.017768093441409505,"tauG":11.343149222800683,"tauS":-11.360917316242093,"tau4":0,"Fs":214.75347736688684,"pe":196.8809358202675,"globalMaxTau2":0.019679624716665955,"globalMaxTau4":0,"globalMaxFs":678.5552779524771,"globalMaxTab":1030.0496259556362,"globalMaxDz":409.3237389579775,"compensationError":0.15664162652204716,"zeta":-43.61013949287524,"zetaApplied":0}},"outputsStale":false}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DP:4</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"dp":4,"name":"Mason CAD (205.3mm Legs) ","color":"none","savedAt":"2026-10-23T01:26:50.770Z","snapshot":{"schema":"general-vsl/v4-pulley","torqueConvention":"physical-link2-ccw/v2","ratioConvention":"output-over-input","parameters":{"L2":200,"L3":200,"ra":50,"rb":25,"rc":35,"rd":35,"re":25,"rf":25,"rw":200,"alpha":20,"phi0":0,"te":100,"tc":165,"m1":8.75,"m2":0,"m3":0,"m5":0,"m6":0,"g":9.81,"beta":0,"Fn":85.8375,"Ft":0,"Fy":0,"Fz":85.8375,"loadMode":"yz","Tab0":0,"Tcd0":0,"Tef0":0,"springEnabled":true,"springK":6,"hornR":62.88850811914982,"Sv":80,"rs":10,"p0":137.88681177871507,"nu":0,"Su":8.418095061266762},"driven":{"q23":"L3","qab":"qab","qdc":"qdc","qfe":"qfe"},"springDriven":null,"springDriving":{"springK":true,"hornR":false,"Sv":true,"rs":true,"p0":false,"nu":true,"Su":false},"ranges":{"alpha":{"min":0,"max":30},"beta":{"min":0,"max":90},"Fn":{"min":0,"max":200},"Ft":{"min":-100,"max":100},"Fy":{"min":-100,"max":100},"Fz":{"min":0,"max":200}},"theta2":149.27616068766133,"period":8,"absoluteTorques":false,"fullTravel":false,"clampRanges":true,"view":{"showTau2":true,"showTau4":true,"showWheelForces":true,"showWheel":true,"showAB":true,"showDrive":true},"visible":{"t3":true,"t5":true,"t6":true,"du":true,"dv":true,"dy":true,"dz":true,"gammaUV":true,"gammaYZ":true},"series":{"t2-torque-tauG":true,"t2-torque-tauS":true,"t2-torque-tau2":true,"t2-torque-tau4":true,"t2-tension-ab":true,"t2-tension-cd":true,"t2-tension-ef":true,"t2-force-F12":true,"t2-force-F14":true,"t2-force-F25":true,"t2-force-F32":true,"t2-force-Fw":true,"dz-torque-tauG":true,"dz-torque-tauS":true,"dz-torque-tau2":true,"dz-torque-tau4":true,"dz-tension-ab":true,"dz-tension-cd":true,"dz-tension-ef":true,"dz-force-F12":true,"dz-force-F14":true,"dz-force-F25":true,"dz-force-F32":true,"dz-force-Fw":true,"beta-torque-tauG":true,"beta-torque-tauS":true,"beta-torque-tau2":true,"beta-torque-tau4":true,"beta-tension-ab":true,"beta-tension-cd":true,"beta-tension-ef":true,"beta-force-F12":true,"beta-force-F14":true,"beta-force-F25":true,"beta-force-F32":true,"beta-force-Fw":true,"alpha-torque-tauG":true,"alpha-torque-tauS":true,"alpha-torque-tau2":true,"alpha-torque-tau4":true,"alpha-tension-ab":true,"alpha-tension-cd":true,"alpha-tension-ef":true,"alpha-force-F12":true,"alpha-force-F14":true,"alpha-force-F25":true,"alpha-force-F32":true,"alpha-force-Fw":true},"outputs":{"tau2":0.015115453537447365,"tauG":27.735715196569537,"tauS":-27.750830650106984,"tau4":0,"Fs":455.8266719381592,"pe":155.87549223213014,"globalMaxTau2":-0.01565360153959716,"globalMaxTau4":17.1675,"globalMaxFs":552.6499900306806,"globalMaxTab":686.6997506370908,"globalMaxDz":272.88249263865174,"compensationError":0.054498156727933456,"zeta":-42.885397396080656,"zetaApplied":0}},"outputsStale":false}</t>
         </is>
       </c>
     </row>

</xml_diff>